<commit_message>
update after day2 PhD
</commit_message>
<xml_diff>
--- a/Eigener Einarbeitungsplan PhD.xlsx
+++ b/Eigener Einarbeitungsplan PhD.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hauke\Desktop\PhD MPSD Bester\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87564B44-4101-4E21-92E4-A4B526BFE0D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{187B98A6-86ED-4189-8A41-617B7357957A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="44">
   <si>
     <t xml:space="preserve">Thema </t>
   </si>
@@ -115,6 +115,48 @@
   </si>
   <si>
     <t xml:space="preserve">week2 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carl Emil Mölsen Exciton in 2D TMDs lesen </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Freiwillig? </t>
+  </si>
+  <si>
+    <t>Bester Empfehlung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spin vally physics </t>
+  </si>
+  <si>
+    <t xml:space="preserve">week 3 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bester internal wiki study </t>
+  </si>
+  <si>
+    <t>week 1-4</t>
+  </si>
+  <si>
+    <t>Quantum Espresso (DFT Introduction program)</t>
+  </si>
+  <si>
+    <t>Bester und Franz empfohlen</t>
+  </si>
+  <si>
+    <t>week1 -4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mx-package AG Bester Introduction by Franz </t>
+  </si>
+  <si>
+    <t>week 5-7</t>
+  </si>
+  <si>
+    <t>week 1 started with Irene and chemserv guy</t>
+  </si>
+  <si>
+    <t>his dissertation</t>
   </si>
 </sst>
 </file>
@@ -447,9 +489,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="5" max="5" width="18.1796875" customWidth="1"/>
     <col min="6" max="6" width="48.36328125" customWidth="1"/>
     <col min="7" max="8" width="27" customWidth="1"/>
     <col min="10" max="10" width="25.54296875" customWidth="1"/>
@@ -464,6 +507,9 @@
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
+      <c r="E1" t="s">
+        <v>31</v>
+      </c>
       <c r="F1" t="s">
         <v>0</v>
       </c>
@@ -499,81 +545,133 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="F4" t="s">
+    <row r="4" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="17.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" t="s">
+        <v>43</v>
+      </c>
+      <c r="H5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="F6" t="s">
         <v>10</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G6" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="F5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="F6" t="s">
-        <v>16</v>
-      </c>
-      <c r="H6" s="1"/>
+      <c r="I6" s="1" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F7" t="s">
+        <v>35</v>
+      </c>
+      <c r="H7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="F8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="F9" t="s">
+        <v>16</v>
+      </c>
+      <c r="H9" s="1"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="F10" t="s">
         <v>14</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H10" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="F8" t="s">
+    <row r="11" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+      <c r="F11" t="s">
         <v>25</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="H11" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="80" x14ac:dyDescent="0.4">
-      <c r="F9" t="s">
+    <row r="12" spans="1:11" ht="80" x14ac:dyDescent="0.4">
+      <c r="F12" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G12" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H12" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="F10" t="s">
+    <row r="13" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="F13" t="s">
         <v>8</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H13" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="F11" t="s">
+    <row r="14" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="F14" t="s">
         <v>6</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H11" t="s">
+      <c r="H14" t="s">
         <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="F15" t="s">
+        <v>33</v>
+      </c>
+      <c r="H15" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="F16" t="s">
+        <v>40</v>
+      </c>
+      <c r="H16" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
PhD_folder commit 25.09.26 after around 2 weeks PhD - mainly research sketch improved
</commit_message>
<xml_diff>
--- a/Eigener Einarbeitungsplan PhD.xlsx
+++ b/Eigener Einarbeitungsplan PhD.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hauke\Desktop\PhD MPSD Bester\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{187B98A6-86ED-4189-8A41-617B7357957A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4501082-702B-4C66-BAF5-34A22BB891F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="56">
   <si>
     <t xml:space="preserve">Thema </t>
   </si>
@@ -81,9 +81,6 @@
     <t>Gute erste Forschungsskizze schreiben</t>
   </si>
   <si>
-    <t xml:space="preserve">week1 </t>
-  </si>
-  <si>
     <t>Woche 1 (15.09-20.09.26)</t>
   </si>
   <si>
@@ -147,16 +144,55 @@
     <t>week1 -4</t>
   </si>
   <si>
-    <t xml:space="preserve">Mx-package AG Bester Introduction by Franz </t>
-  </si>
-  <si>
     <t>week 5-7</t>
   </si>
   <si>
-    <t>week 1 started with Irene and chemserv guy</t>
-  </si>
-  <si>
     <t>his dissertation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configuration interaction and electronic structure methods </t>
+  </si>
+  <si>
+    <t>week1 -3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quantum chemistry introduction </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mx-package AG Bester Introduction by Franz and code understanding </t>
+  </si>
+  <si>
+    <t>before first draft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">before started </t>
+  </si>
+  <si>
+    <t xml:space="preserve">installed but not run in week1; </t>
+  </si>
+  <si>
+    <t xml:space="preserve">week1: started reading and focused at DFT theory and CI but CI not understood; </t>
+  </si>
+  <si>
+    <t xml:space="preserve">borrowed books in week1 and fast going through one whole introductory book in week1;  </t>
+  </si>
+  <si>
+    <t>week 1 started with Irene and chemserv guy; most programs installed in week1</t>
+  </si>
+  <si>
+    <t>week 2-4</t>
+  </si>
+  <si>
+    <t>no time in week1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">introduction to DFT with Nilelsen dissertation inweek1 and well understood; </t>
+  </si>
+  <si>
+    <t>week2-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reading about CI in Nielsen dissertation but not understood; </t>
   </si>
 </sst>
 </file>
@@ -489,12 +525,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="5" max="5" width="18.1796875" customWidth="1"/>
     <col min="6" max="6" width="48.36328125" customWidth="1"/>
     <col min="7" max="8" width="27" customWidth="1"/>
+    <col min="9" max="9" width="33.7265625" customWidth="1"/>
     <col min="10" max="10" width="25.54296875" customWidth="1"/>
     <col min="11" max="11" width="12.90625" customWidth="1"/>
     <col min="12" max="12" width="15.26953125" customWidth="1"/>
@@ -502,13 +539,13 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F1" t="s">
         <v>0</v>
@@ -534,7 +571,10 @@
         <v>17</v>
       </c>
       <c r="H2" t="s">
-        <v>28</v>
+        <v>27</v>
+      </c>
+      <c r="I2" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
@@ -542,136 +582,174 @@
         <v>5</v>
       </c>
       <c r="H3" t="s">
-        <v>21</v>
+        <v>20</v>
+      </c>
+      <c r="I3" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="H4" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="H4" t="s">
-        <v>39</v>
+      <c r="I4" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="17.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G5" t="s">
+        <v>40</v>
+      </c>
+      <c r="H5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="F6" t="s">
         <v>43</v>
       </c>
-      <c r="H5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="F6" t="s">
+      <c r="H6" t="s">
+        <v>35</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="F8" t="s">
         <v>10</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G8" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="F7" t="s">
-        <v>35</v>
-      </c>
-      <c r="H7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="F8" t="s">
-        <v>22</v>
-      </c>
-      <c r="H8" t="s">
-        <v>23</v>
+      <c r="H8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F9" t="s">
-        <v>16</v>
-      </c>
-      <c r="H9" s="1"/>
+        <v>34</v>
+      </c>
+      <c r="H9" t="s">
+        <v>51</v>
+      </c>
+      <c r="I9" s="1"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F10" t="s">
+        <v>21</v>
+      </c>
+      <c r="H10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="F11" t="s">
+        <v>16</v>
+      </c>
+      <c r="H11" s="1"/>
+    </row>
+    <row r="12" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="F12" t="s">
         <v>14</v>
       </c>
-      <c r="H10" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="F11" t="s">
+      <c r="H12" t="s">
+        <v>19</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+      <c r="F13" t="s">
+        <v>24</v>
+      </c>
+      <c r="G13" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="G11" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="80" x14ac:dyDescent="0.4">
-      <c r="F12" t="s">
+      <c r="H13" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="80" x14ac:dyDescent="0.4">
+      <c r="F14" t="s">
         <v>13</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="G14" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H12" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="F13" t="s">
+      <c r="H14" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="F15" t="s">
         <v>8</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="H13" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="F14" t="s">
+      <c r="H15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="F16" t="s">
         <v>6</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H14" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="F15" t="s">
+      <c r="H16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="6:9" x14ac:dyDescent="0.35">
+      <c r="F17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H17" t="s">
         <v>33</v>
       </c>
-      <c r="H15" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="F16" t="s">
-        <v>40</v>
-      </c>
-      <c r="H16" t="s">
+    </row>
+    <row r="18" spans="6:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="F18" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H18" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="19" spans="6:9" x14ac:dyDescent="0.35">
+      <c r="F19" t="s">
         <v>41</v>
+      </c>
+      <c r="H19" t="s">
+        <v>42</v>
+      </c>
+      <c r="I19" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
PhD directory at 7.10.26 3.5 weeks after start
</commit_message>
<xml_diff>
--- a/Eigener Einarbeitungsplan PhD.xlsx
+++ b/Eigener Einarbeitungsplan PhD.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hauke\Desktop\PhD MPSD Bester\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4501082-702B-4C66-BAF5-34A22BB891F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C74D3031-FA86-4D4C-B978-C43C1D7FBED8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="65">
   <si>
     <t xml:space="preserve">Thema </t>
   </si>
@@ -162,21 +162,6 @@
     <t xml:space="preserve">Mx-package AG Bester Introduction by Franz and code understanding </t>
   </si>
   <si>
-    <t>before first draft</t>
-  </si>
-  <si>
-    <t xml:space="preserve">before started </t>
-  </si>
-  <si>
-    <t xml:space="preserve">installed but not run in week1; </t>
-  </si>
-  <si>
-    <t xml:space="preserve">week1: started reading and focused at DFT theory and CI but CI not understood; </t>
-  </si>
-  <si>
-    <t xml:space="preserve">borrowed books in week1 and fast going through one whole introductory book in week1;  </t>
-  </si>
-  <si>
     <t>week 1 started with Irene and chemserv guy; most programs installed in week1</t>
   </si>
   <si>
@@ -186,13 +171,55 @@
     <t>no time in week1</t>
   </si>
   <si>
-    <t xml:space="preserve">introduction to DFT with Nilelsen dissertation inweek1 and well understood; </t>
-  </si>
-  <si>
     <t>week2-5</t>
   </si>
   <si>
-    <t xml:space="preserve">reading about CI in Nielsen dissertation but not understood; </t>
+    <t>before first draft, much more precise second draft with integration in group work in week2, send to G. Bester</t>
+  </si>
+  <si>
+    <t>before and week 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">before started, not really improved in week 1 and 2 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">week1: started reading and focused at DFT theory and CI but CI not understood; week2: reading roughly about his papers (abstract, introduction, conclusion); </t>
+  </si>
+  <si>
+    <t>borrowed books in week1 and fast going through one whole introductory book in week1;  general concepts googled in week2</t>
+  </si>
+  <si>
+    <t>introduction to DFT with Nilelsen dissertation inweek1 and well understood; watched Quantum esprresso video with DFT in week2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">week1: reading a bit about CI in Nielsen dissertation but not understood; </t>
+  </si>
+  <si>
+    <t>week 3-8</t>
+  </si>
+  <si>
+    <t>Book Essentials of Computational Chemistry reading</t>
+  </si>
+  <si>
+    <t>installed but not run in week1 and 2; watched introductory video about QE in week 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">problems with getting access to clusterand finding login node in week 1 and 2 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Introduction many body quantum physics </t>
+  </si>
+  <si>
+    <t>long lecture script</t>
+  </si>
+  <si>
+    <t>not finished in week2 but in week3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salted machine learning learning </t>
+  </si>
+  <si>
+    <t xml:space="preserve">week5 </t>
   </si>
 </sst>
 </file>
@@ -525,15 +552,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="5" max="5" width="18.1796875" customWidth="1"/>
     <col min="6" max="6" width="48.36328125" customWidth="1"/>
     <col min="7" max="8" width="27" customWidth="1"/>
     <col min="9" max="9" width="33.7265625" customWidth="1"/>
-    <col min="10" max="10" width="25.54296875" customWidth="1"/>
-    <col min="11" max="11" width="12.90625" customWidth="1"/>
+    <col min="10" max="10" width="31.26953125" customWidth="1"/>
+    <col min="11" max="11" width="18.6328125" customWidth="1"/>
     <col min="12" max="12" width="15.26953125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -566,29 +593,35 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="F2" t="s">
         <v>17</v>
       </c>
       <c r="H2" t="s">
         <v>27</v>
       </c>
-      <c r="I2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="I2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="J2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="F3" t="s">
         <v>5</v>
       </c>
       <c r="H3" t="s">
         <v>20</v>
       </c>
-      <c r="I3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="I3" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E4" s="1" t="s">
         <v>37</v>
       </c>
@@ -598,11 +631,14 @@
       <c r="H4" t="s">
         <v>38</v>
       </c>
-      <c r="I4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="17.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="I4" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="80" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E5" t="s">
         <v>31</v>
       </c>
@@ -613,13 +649,13 @@
         <v>40</v>
       </c>
       <c r="H5" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="F6" t="s">
         <v>43</v>
       </c>
@@ -627,7 +663,18 @@
         <v>35</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>49</v>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="F7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G7" t="s">
+        <v>61</v>
+      </c>
+      <c r="H7" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -641,7 +688,7 @@
         <v>18</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
@@ -649,7 +696,7 @@
         <v>34</v>
       </c>
       <c r="H9" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="I9" s="1"/>
     </row>
@@ -661,7 +708,7 @@
         <v>22</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
@@ -670,7 +717,7 @@
       </c>
       <c r="H11" s="1"/>
     </row>
-    <row r="12" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="F12" t="s">
         <v>14</v>
       </c>
@@ -678,7 +725,7 @@
         <v>19</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="58" x14ac:dyDescent="0.35">
@@ -700,7 +747,7 @@
         <v>15</v>
       </c>
       <c r="H14" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -741,15 +788,31 @@
         <v>39</v>
       </c>
     </row>
-    <row r="19" spans="6:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="6:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="F19" t="s">
         <v>41</v>
       </c>
       <c r="H19" t="s">
         <v>42</v>
       </c>
-      <c r="I19" t="s">
+      <c r="I19" s="1" t="s">
         <v>55</v>
+      </c>
+    </row>
+    <row r="20" spans="6:9" x14ac:dyDescent="0.35">
+      <c r="F20" t="s">
+        <v>57</v>
+      </c>
+      <c r="H20" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21" spans="6:9" x14ac:dyDescent="0.35">
+      <c r="F21" t="s">
+        <v>63</v>
+      </c>
+      <c r="H21" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>